<commit_message>
content: founder access decisions — two free samples, Saturn featured
Founder decisions 2026-08-16: the free tier samples are the-rings-of-
saturn and the-bakery-before-dawn (bakery flips premium->free, matching
the row already published free in staging); every other story is
premium, resolving the two PENDING access decisions (the-bay-that-
glows-at-night, the-clockmaker-s-workshop); Saturn is the featured
story. All changes made in story.yaml and regenerated via lullable.py
build + tracker; Saturn re-validates PUBLISH READY on all 17 gates.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Lullable_Story_Card_Tracker.xlsx
+++ b/Lullable_Story_Card_Tracker.xlsx
@@ -1759,7 +1759,7 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>premium</t>
+          <t>free</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
@@ -1978,7 +1978,7 @@
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>premium</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
@@ -2169,7 +2169,7 @@
       </c>
       <c r="AQ9" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AR9" s="9" t="inlineStr">
@@ -2416,7 +2416,7 @@
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>premium</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
@@ -2607,7 +2607,7 @@
       </c>
       <c r="AQ11" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AR11" s="9" t="inlineStr">
@@ -4423,7 +4423,7 @@
       </c>
       <c r="L20" s="7" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="M20" s="7" t="inlineStr">

</xml_diff>

<commit_message>
content: adopt the three legacy staging rows into the manifest pipeline (D27)
Executes app-repo DECISIONS.md §19 (founder 2026-08-16): aristotle (free) and
dinosaurs (premium) adopted rather than archived; bakery's manifest catches up
with its 2026-08-16 free staging publication.

All audio blocks computed by closeout from real bytes; the re-encoded delivery
files are byte-identical to the uploaded staging assets (sha256 match). All
three at workflowStatus: staging with honest gaps: G12/G07 render provenance,
G13 QA sign-off, and G17 narration text for the two legacy episodes.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Lullable_Story_Card_Tracker.xlsx
+++ b/Lullable_Story_Card_Tracker.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Story Tracker" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Story Tracker'!$A$3:$AS$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Story Tracker'!$A$3:$AS$24</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -562,7 +562,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AS22"/>
+  <dimension ref="A1:AS24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1310,43 +1310,43 @@
     <row r="6" ht="26" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>floating-through-the-pillars-of-creation</t>
+          <t>aristotle-the-greatest-philosopher</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr"/>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>staging</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>premium</t>
+          <t>free</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>free</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>Floating Through the Pillars of Creation</t>
+          <t>Aristotle, the Greatest Philosopher</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>Cold columns of dust and gas, six thousand light years out, quietly making stars</t>
+          <t>A quiet journey through reason, virtue, and the good life</t>
         </is>
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>Lullable</t>
+          <t>Andrew</t>
         </is>
       </c>
       <c r="I6" s="7" t="inlineStr">
         <is>
-          <t>cosmic-journeys</t>
+          <t>ancient-worlds</t>
         </is>
       </c>
       <c r="J6" s="7" t="inlineStr"/>
@@ -1362,57 +1362,55 @@
       </c>
       <c r="M6" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>2026-08-09T00:00:00Z</t>
         </is>
       </c>
       <c r="N6" s="7" t="inlineStr">
         <is>
-          <t>1A1026</t>
+          <t>26384A</t>
         </is>
       </c>
       <c r="O6" s="7" t="inlineStr">
         <is>
-          <t>C98A6B</t>
-        </is>
-      </c>
-      <c r="P6" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
+          <t>B89A6A</t>
+        </is>
+      </c>
+      <c r="P6" s="8" t="n">
+        <v>2640</v>
       </c>
       <c r="Q6" s="7" t="inlineStr">
         <is>
-          <t>Nothing out there is waiting for anything. The columns simply stand in the light, giving themselves up to it slowly, and they will go on standing long after tonight.</t>
+          <t>One calm mind, examined slowly — reason, virtue, and the good life, laid out like a quiet evening walk. Nothing here needs to be solved tonight.</t>
         </is>
       </c>
       <c r="R6" s="7" t="inlineStr">
         <is>
-          <t>Feeling small and safe</t>
+          <t>Curious, wandering minds</t>
         </is>
       </c>
       <c r="S6" s="7" t="inlineStr">
         <is>
-          <t>Slow and drifting</t>
+          <t>Slow and steady</t>
         </is>
       </c>
       <c r="T6" s="7" t="inlineStr">
         <is>
-          <t>Cold, dusty, lit from above</t>
+          <t>Marble, lamplight, reason</t>
         </is>
       </c>
       <c r="U6" s="7" t="inlineStr">
         <is>
-          <t>You rise from your own roof and travel outward, past every planet, until the stars themselves begin to thicken into a glowing cloud. Three dark columns stand in the middle of it, each one taller than the gap between our sun and its nearest neighbour. You learn what they are made of, how starlight is quietly carving them, why they are pillars at all, and what is forming in the pockets of shadow inside. Then the light goes on arriving, as it has for six thousand years, and you let all of it go.</t>
+          <t>You settle in beside one of history’s calmest minds. This is a slow exploration of Aristotle’s life and ideas — how he watched the natural world, what he taught about knowledge, character, and friendship, and why his patient way of thinking still shapes how we understand ourselves. The questions are old, the pace is gentle, and nothing needs deciding tonight.</t>
         </is>
       </c>
       <c r="V6" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>audio-aristotle-en-v1-aac96</t>
         </is>
       </c>
       <c r="W6" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>master.wav</t>
         </is>
       </c>
       <c r="X6" s="7" t="inlineStr">
@@ -1427,7 +1425,7 @@
       </c>
       <c r="Z6" s="9" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>staging</t>
         </is>
       </c>
       <c r="AA6" s="9" t="inlineStr">
@@ -1462,7 +1460,7 @@
       </c>
       <c r="AG6" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AH6" s="9" t="inlineStr">
@@ -1472,22 +1470,22 @@
       </c>
       <c r="AI6" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AJ6" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AK6" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AL6" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AM6" s="9" t="inlineStr">
@@ -1502,7 +1500,7 @@
       </c>
       <c r="AO6" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AP6" s="9" t="inlineStr">
@@ -1517,25 +1515,25 @@
       </c>
       <c r="AR6" s="9" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="AS6" s="9" t="inlineStr">
         <is>
-          <t>Stories/floating-through-the-pillars-of-creation/story.yaml</t>
+          <t>Stories/aristotle-the-greatest-philosopher/story.yaml</t>
         </is>
       </c>
     </row>
     <row r="7" ht="26" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>mapping-the-cosmic-web</t>
+          <t>dinosaurs-from-rule-to-ruin</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr"/>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>staging</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
@@ -1545,27 +1543,27 @@
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>premium</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>Mapping the Cosmic Web</t>
+          <t>The Dinosaurs: From Rule to Ruin</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>Decades of cold nights on mountains, one galaxy at a time, until a shape appeared</t>
+          <t>A 44-minute journey through deep time</t>
         </is>
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>Lullable</t>
+          <t>Sleep Stories by AVP</t>
         </is>
       </c>
       <c r="I7" s="7" t="inlineStr">
         <is>
-          <t>cosmic-journeys</t>
+          <t>ancient-worlds</t>
         </is>
       </c>
       <c r="J7" s="7" t="inlineStr"/>
@@ -1581,57 +1579,55 @@
       </c>
       <c r="M7" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>2026-08-11T02:11:43Z</t>
         </is>
       </c>
       <c r="N7" s="7" t="inlineStr">
         <is>
-          <t>10131F</t>
+          <t>26384A</t>
         </is>
       </c>
       <c r="O7" s="7" t="inlineStr">
         <is>
-          <t>8E9FD0</t>
-        </is>
-      </c>
-      <c r="P7" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
+          <t>B89A6A</t>
+        </is>
+      </c>
+      <c r="P7" s="8" t="n">
+        <v>2690</v>
       </c>
       <c r="Q7" s="7" t="inlineStr">
         <is>
-          <t>The largest arrangement there is, and it does nothing in any hurry. It was found by people writing down one number a night, and none of it needs your attention tonight.</t>
+          <t>Deep time moves slowly here. Every age in this story settled into stillness long ago, and nothing in it asks anything of you tonight.</t>
         </is>
       </c>
       <c r="R7" s="7" t="inlineStr">
         <is>
-          <t>Ending a long day</t>
+          <t>Drifting through time</t>
         </is>
       </c>
       <c r="S7" s="7" t="inlineStr">
         <is>
-          <t>Slow, wide, still</t>
+          <t>Slow and steady</t>
         </is>
       </c>
       <c r="T7" s="7" t="inlineStr">
         <is>
-          <t>Vast, dark, quiet, patient</t>
+          <t>Ancient, vast, hushed</t>
         </is>
       </c>
       <c r="U7" s="7" t="inlineStr">
         <is>
-          <t>Sit in a cold dome in Arizona in the 1980s, while somebody points a telescope at one faint smudge after another and writes down a number. Do that for years, plot the results, and a shape appears that nobody expected — galaxies strung along threads, gathered at knots, wrapped around enormous quiet rooms with almost nothing inside. Along the way, the mule driver who became one of the great observers, a sound from the early universe frozen into the sky as a ruler, and five thousand small robots that rearrange themselves in the dark.</t>
+          <t>Drift through the rise, reign, and quiet fading of the dinosaurs in a calm story of deep time. You move slowly across changing continents and warm shallow seas, through long ages when giants grazed in the light of an older sun, and follow the traces they left behind in stone — a world that never fully ended, still with us in every morning’s birdsong.</t>
         </is>
       </c>
       <c r="V7" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>audio-dinosaurs-en-v1-aac96</t>
         </is>
       </c>
       <c r="W7" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>master.wav</t>
         </is>
       </c>
       <c r="X7" s="7" t="inlineStr">
@@ -1646,7 +1642,7 @@
       </c>
       <c r="Z7" s="9" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>staging</t>
         </is>
       </c>
       <c r="AA7" s="9" t="inlineStr">
@@ -1681,7 +1677,7 @@
       </c>
       <c r="AG7" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AH7" s="9" t="inlineStr">
@@ -1691,22 +1687,22 @@
       </c>
       <c r="AI7" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AJ7" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AK7" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AL7" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AM7" s="9" t="inlineStr">
@@ -1721,7 +1717,7 @@
       </c>
       <c r="AO7" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AP7" s="9" t="inlineStr">
@@ -1736,19 +1732,19 @@
       </c>
       <c r="AR7" s="9" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="AS7" s="9" t="inlineStr">
         <is>
-          <t>Stories/mapping-the-cosmic-web/story.yaml</t>
+          <t>Stories/dinosaurs-from-rule-to-ruin/story.yaml</t>
         </is>
       </c>
     </row>
     <row r="8" ht="26" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>the-bakery-before-dawn</t>
+          <t>floating-through-the-pillars-of-creation</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr"/>
@@ -1759,7 +1755,7 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>free</t>
+          <t>premium</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
@@ -1769,12 +1765,12 @@
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>The Bakery Before Dawn</t>
+          <t>Floating Through the Pillars of Creation</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>Warm flour, a slow rising, and the long quiet hours before a town wakes</t>
+          <t>Cold columns of dust and gas, six thousand light years out, quietly making stars</t>
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr">
@@ -1784,7 +1780,7 @@
       </c>
       <c r="I8" s="7" t="inlineStr">
         <is>
-          <t>cozy-tales</t>
+          <t>cosmic-journeys</t>
         </is>
       </c>
       <c r="J8" s="7" t="inlineStr"/>
@@ -1805,12 +1801,12 @@
       </c>
       <c r="N8" s="7" t="inlineStr">
         <is>
-          <t>2E1F14</t>
+          <t>1A1026</t>
         </is>
       </c>
       <c r="O8" s="7" t="inlineStr">
         <is>
-          <t>E3B778</t>
+          <t>C98A6B</t>
         </is>
       </c>
       <c r="P8" s="8" t="inlineStr">
@@ -1820,27 +1816,27 @@
       </c>
       <c r="Q8" s="7" t="inlineStr">
         <is>
-          <t>Someone else is already awake, working gently in the warm, at something that cannot be hurried. There is nothing here you need to do.</t>
+          <t>Nothing out there is waiting for anything. The columns simply stand in the light, giving themselves up to it slowly, and they will go on standing long after tonight.</t>
         </is>
       </c>
       <c r="R8" s="7" t="inlineStr">
         <is>
-          <t>Feeling safe and warm</t>
+          <t>Feeling small and safe</t>
         </is>
       </c>
       <c r="S8" s="7" t="inlineStr">
         <is>
-          <t>Slow and steady</t>
+          <t>Slow and drifting</t>
         </is>
       </c>
       <c r="T8" s="7" t="inlineStr">
         <is>
-          <t>Warm, floury, hushed</t>
+          <t>Cold, dusty, lit from above</t>
         </is>
       </c>
       <c r="U8" s="7" t="inlineStr">
         <is>
-          <t>You cross a frozen street at two in the morning toward the one lit window on the corner, and step into a small tiled room that smells of warm flour. A baker works alone at a wooden bench, unhurried, feeding a glass jar that is older than she is. You learn what is living inside it, why the dough rests before it is touched, what the salt is quietly doing, and how a loaf lifts and sets and turns gold in the last half hour. Then the light goes off, and she walks home to sleep.</t>
+          <t>You rise from your own roof and travel outward, past every planet, until the stars themselves begin to thicken into a glowing cloud. Three dark columns stand in the middle of it, each one taller than the gap between our sun and its nearest neighbour. You learn what they are made of, how starlight is quietly carving them, why they are pillars at all, and what is forming in the pockets of shadow inside. Then the light goes on arriving, as it has for six thousand years, and you let all of it go.</t>
         </is>
       </c>
       <c r="V8" s="7" t="inlineStr">
@@ -1960,14 +1956,14 @@
       </c>
       <c r="AS8" s="9" t="inlineStr">
         <is>
-          <t>Stories/the-bakery-before-dawn/story.yaml</t>
+          <t>Stories/floating-through-the-pillars-of-creation/story.yaml</t>
         </is>
       </c>
     </row>
     <row r="9" ht="26" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>the-bay-that-glows-at-night</t>
+          <t>mapping-the-cosmic-web</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr"/>
@@ -1988,12 +1984,12 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>The Bay That Glows at Night</t>
+          <t>Mapping the Cosmic Web</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>Adrift on a moonless Caribbean bay where every touch of the water answers in blue</t>
+          <t>Decades of cold nights on mountains, one galaxy at a time, until a shape appeared</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr">
@@ -2003,7 +1999,7 @@
       </c>
       <c r="I9" s="7" t="inlineStr">
         <is>
-          <t>gentle-nature</t>
+          <t>cosmic-journeys</t>
         </is>
       </c>
       <c r="J9" s="7" t="inlineStr"/>
@@ -2024,12 +2020,12 @@
       </c>
       <c r="N9" s="7" t="inlineStr">
         <is>
-          <t>0A1622</t>
+          <t>10131F</t>
         </is>
       </c>
       <c r="O9" s="7" t="inlineStr">
         <is>
-          <t>63D9F2</t>
+          <t>8E9FD0</t>
         </is>
       </c>
       <c r="P9" s="8" t="inlineStr">
@@ -2039,27 +2035,27 @@
       </c>
       <c r="Q9" s="7" t="inlineStr">
         <is>
-          <t>No moon tonight, and that is the point. The paddle rests, the water glows wherever the fish go, and a whole island keeps its darkness like a garden.</t>
+          <t>The largest arrangement there is, and it does nothing in any hurry. It was found by people writing down one number a night, and none of it needs your attention tonight.</t>
         </is>
       </c>
       <c r="R9" s="7" t="inlineStr">
         <is>
-          <t>Dimming a busy mind</t>
+          <t>Ending a long day</t>
         </is>
       </c>
       <c r="S9" s="7" t="inlineStr">
         <is>
-          <t>Adrift and moonless</t>
+          <t>Slow, wide, still</t>
         </is>
       </c>
       <c r="T9" s="7" t="inlineStr">
         <is>
-          <t>Warm dark, blue sparks</t>
+          <t>Vast, dark, quiet, patient</t>
         </is>
       </c>
       <c r="U9" s="7" t="inlineStr">
         <is>
-          <t>Glide out through a tunnel of mangroves onto the brightest glowing bay in the world, on a night with no moon. Learn how a single living cell, one of seven hundred thousand in every gallon, keeps a tiny pantry of light and opens it at a touch. Watch fish write comet trails, hold a handful of blue stars, and float between two skies while warm rain sets the whole surface flickering. With Darwin at the ship's rail, the rare milky seas that glow from horizon to horizon, and an island community that tends its darkness the way other towns tend their gardens.</t>
+          <t>Sit in a cold dome in Arizona in the 1980s, while somebody points a telescope at one faint smudge after another and writes down a number. Do that for years, plot the results, and a shape appears that nobody expected — galaxies strung along threads, gathered at knots, wrapped around enormous quiet rooms with almost nothing inside. Along the way, the mule driver who became one of the great observers, a sound from the early universe frozen into the sky as a ruler, and five thousand small robots that rearrange themselves in the dark.</t>
         </is>
       </c>
       <c r="V9" s="7" t="inlineStr">
@@ -2179,40 +2175,40 @@
       </c>
       <c r="AS9" s="9" t="inlineStr">
         <is>
-          <t>Stories/the-bay-that-glows-at-night/story.yaml</t>
+          <t>Stories/mapping-the-cosmic-web/story.yaml</t>
         </is>
       </c>
     </row>
     <row r="10" ht="26" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>the-building-of-a-cathedral</t>
+          <t>the-bakery-before-dawn</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr"/>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>staging</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>premium</t>
+          <t>free</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>free</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>The Building of a Cathedral</t>
+          <t>The Bakery Before Dawn</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>An evening among people entirely at peace with never finishing</t>
+          <t>Warm flour, a slow rising, and the long quiet hours before a town wakes</t>
         </is>
       </c>
       <c r="H10" s="7" t="inlineStr">
@@ -2222,7 +2218,7 @@
       </c>
       <c r="I10" s="7" t="inlineStr">
         <is>
-          <t>ancient-worlds</t>
+          <t>cozy-tales</t>
         </is>
       </c>
       <c r="J10" s="7" t="inlineStr"/>
@@ -2238,57 +2234,55 @@
       </c>
       <c r="M10" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>2026-08-16T15:26:08Z</t>
         </is>
       </c>
       <c r="N10" s="7" t="inlineStr">
         <is>
-          <t>26222B</t>
+          <t>2E1F14</t>
         </is>
       </c>
       <c r="O10" s="7" t="inlineStr">
         <is>
-          <t>C9A2C8</t>
-        </is>
-      </c>
-      <c r="P10" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
+          <t>E3B778</t>
+        </is>
+      </c>
+      <c r="P10" s="8" t="n">
+        <v>2174</v>
       </c>
       <c r="Q10" s="7" t="inlineStr">
         <is>
-          <t>Sixty years done, eighty to go, and every person on the site content with that arithmetic. Nothing in your life needs finishing by morning either.</t>
+          <t>Someone else is already awake, working gently in the warm, at something that cannot be hurried. There is nothing here you need to do.</t>
         </is>
       </c>
       <c r="R10" s="7" t="inlineStr">
         <is>
-          <t>Setting worries down</t>
+          <t>Feeling safe and warm</t>
         </is>
       </c>
       <c r="S10" s="7" t="inlineStr">
         <is>
-          <t>Generational and calm</t>
+          <t>Slow and steady</t>
         </is>
       </c>
       <c r="T10" s="7" t="inlineStr">
         <is>
-          <t>Stone, dusk, gold, chant</t>
+          <t>Warm, floury, hushed</t>
         </is>
       </c>
       <c r="U10" s="7" t="inlineStr">
         <is>
-          <t>Walk into a thirteenth-century city at dusk, where the largest unfinished thing in the world has been rising for sixty years and will not be done for eighty more. Visit the lodge where stone dust turns gold in the doorway light, and the plaster tracing floor where three generations of masters have scratched their thinking at full size. Learn why the pointed arch lets stone float, how a timber centering is struck and a vault suddenly holds itself, and why lime mortar sets the pace of the whole century. Then watch the site put itself to bed, wrapped in straw against the frost, still quietly turning back into stone in the dark.</t>
+          <t>You cross a frozen street at two in the morning toward the one lit window on the corner, and step into a small tiled room that smells of warm flour. A baker works alone at a wooden bench, unhurried, feeding a glass jar that is older than she is. You learn what is living inside it, why the dough rests before it is touched, what the salt is quietly doing, and how a loaf lifts and sets and turns gold in the last half hour. Then the light goes off, and she walks home to sleep.</t>
         </is>
       </c>
       <c r="V10" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>audio-the-bakery-before-dawn-en-v1-aac96</t>
         </is>
       </c>
       <c r="W10" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>ElevenLabs_the-bakery-before-dawn.wav</t>
         </is>
       </c>
       <c r="X10" s="7" t="inlineStr">
@@ -2303,7 +2297,7 @@
       </c>
       <c r="Z10" s="9" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>staging</t>
         </is>
       </c>
       <c r="AA10" s="9" t="inlineStr">
@@ -2338,7 +2332,7 @@
       </c>
       <c r="AG10" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AH10" s="9" t="inlineStr">
@@ -2348,22 +2342,22 @@
       </c>
       <c r="AI10" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AJ10" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AK10" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AL10" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AM10" s="9" t="inlineStr">
@@ -2378,7 +2372,7 @@
       </c>
       <c r="AO10" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AP10" s="9" t="inlineStr">
@@ -2398,14 +2392,14 @@
       </c>
       <c r="AS10" s="9" t="inlineStr">
         <is>
-          <t>Stories/the-building-of-a-cathedral/story.yaml</t>
+          <t>Stories/the-bakery-before-dawn/story.yaml</t>
         </is>
       </c>
     </row>
     <row r="11" ht="26" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>the-clockmaker-s-workshop</t>
+          <t>the-bay-that-glows-at-night</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr"/>
@@ -2426,12 +2420,12 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>The Clockmaker's Workshop</t>
+          <t>The Bay That Glows at Night</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>An evening among a hundred gentle clocks, none of them quite in agreement</t>
+          <t>Adrift on a moonless Caribbean bay where every touch of the water answers in blue</t>
         </is>
       </c>
       <c r="H11" s="7" t="inlineStr">
@@ -2441,7 +2435,7 @@
       </c>
       <c r="I11" s="7" t="inlineStr">
         <is>
-          <t>cozy-tales</t>
+          <t>gentle-nature</t>
         </is>
       </c>
       <c r="J11" s="7" t="inlineStr"/>
@@ -2462,12 +2456,12 @@
       </c>
       <c r="N11" s="7" t="inlineStr">
         <is>
-          <t>1C140E</t>
+          <t>0A1622</t>
         </is>
       </c>
       <c r="O11" s="7" t="inlineStr">
         <is>
-          <t>C98F3D</t>
+          <t>63D9F2</t>
         </is>
       </c>
       <c r="P11" s="8" t="inlineStr">
@@ -2477,27 +2471,27 @@
       </c>
       <c r="Q11" s="7" t="inlineStr">
         <is>
-          <t>The shop is locked, the lamp is out, and every pendulum keeps its small agreement in the dark. Nobody has to keep time while they sleep. It is being handled.</t>
+          <t>No moon tonight, and that is the point. The paddle rests, the water glows wherever the fish go, and a whole island keeps its darkness like a garden.</t>
         </is>
       </c>
       <c r="R11" s="7" t="inlineStr">
         <is>
-          <t>Ticking down to rest</t>
+          <t>Dimming a busy mind</t>
         </is>
       </c>
       <c r="S11" s="7" t="inlineStr">
         <is>
-          <t>Once a second, forever</t>
+          <t>Adrift and moonless</t>
         </is>
       </c>
       <c r="T11" s="7" t="inlineStr">
         <is>
-          <t>Brass, oil, a hundred ticks</t>
+          <t>Warm dark, blue sparks</t>
         </is>
       </c>
       <c r="U11" s="7" t="inlineStr">
         <is>
-          <t>Step through a door with a brass bell into a small-town shop where a hundred clocks tick softly out of step, like rain on a roof. At the bench, an unhurried craftsman tends a movement of polished wheels with tools that have not changed in two centuries. Learn what a clock really is, a falling weight let down slowly over a week, and why two clocks on the same wall drift into perfect step with each other, a mystery first noticed from a sickbed in 1665. With painted moon dials, a drawer of orphaned keys that all fit something somewhere, winding day, house calls taken over tea, and the repairers' names penciled inside case doors, a century apart.</t>
+          <t>Glide out through a tunnel of mangroves onto the brightest glowing bay in the world, on a night with no moon. Learn how a single living cell, one of seven hundred thousand in every gallon, keeps a tiny pantry of light and opens it at a touch. Watch fish write comet trails, hold a handful of blue stars, and float between two skies while warm rain sets the whole surface flickering. With Darwin at the ship's rail, the rare milky seas that glow from horizon to horizon, and an island community that tends its darkness the way other towns tend their gardens.</t>
         </is>
       </c>
       <c r="V11" s="7" t="inlineStr">
@@ -2617,14 +2611,14 @@
       </c>
       <c r="AS11" s="9" t="inlineStr">
         <is>
-          <t>Stories/the-clockmaker-s-workshop/story.yaml</t>
+          <t>Stories/the-bay-that-glows-at-night/story.yaml</t>
         </is>
       </c>
     </row>
     <row r="12" ht="26" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>the-deep-ocean-trenches</t>
+          <t>the-building-of-a-cathedral</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr"/>
@@ -2645,22 +2639,22 @@
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>The Deep Ocean Trenches</t>
+          <t>The Building of a Cathedral</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>A slow descent past the last of the light, into the stillest water on earth</t>
+          <t>An evening among people entirely at peace with never finishing</t>
         </is>
       </c>
       <c r="H12" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>Lullable</t>
         </is>
       </c>
       <c r="I12" s="7" t="inlineStr">
         <is>
-          <t>gentle-nature</t>
+          <t>ancient-worlds</t>
         </is>
       </c>
       <c r="J12" s="7" t="inlineStr"/>
@@ -2681,12 +2675,12 @@
       </c>
       <c r="N12" s="7" t="inlineStr">
         <is>
-          <t>0B1F33</t>
+          <t>26222B</t>
         </is>
       </c>
       <c r="O12" s="7" t="inlineStr">
         <is>
-          <t>5FA8C4</t>
+          <t>C9A2C8</t>
         </is>
       </c>
       <c r="P12" s="8" t="inlineStr">
@@ -2696,27 +2690,27 @@
       </c>
       <c r="Q12" s="7" t="inlineStr">
         <is>
-          <t>One slow direction, downward, and nothing waiting at the end of it. An easy thing to follow, and an easier thing to let go of.</t>
+          <t>Sixty years done, eighty to go, and every person on the site content with that arithmetic. Nothing in your life needs finishing by morning either.</t>
         </is>
       </c>
       <c r="R12" s="7" t="inlineStr">
         <is>
-          <t>Letting the day end</t>
+          <t>Setting worries down</t>
         </is>
       </c>
       <c r="S12" s="7" t="inlineStr">
         <is>
-          <t>Slow and sinking</t>
+          <t>Generational and calm</t>
         </is>
       </c>
       <c r="T12" s="7" t="inlineStr">
         <is>
-          <t>Dark, cool, weightless</t>
+          <t>Stone, dusk, gold, chant</t>
         </is>
       </c>
       <c r="U12" s="7" t="inlineStr">
         <is>
-          <t>You slip beneath a starlit sea and sink, without effort, through the sunlit water and the long blue twilight into a darkness the sun has never reached. Small living lights blink on and drift away. Marine snow falls, soft and endless, all the way down to a floor of pale sediment older than memory. Further down still lie the trenches, where the pressure feels only like stillness and there is nowhere deeper to go.</t>
+          <t>Walk into a thirteenth-century city at dusk, where the largest unfinished thing in the world has been rising for sixty years and will not be done for eighty more. Visit the lodge where stone dust turns gold in the doorway light, and the plaster tracing floor where three generations of masters have scratched their thinking at full size. Learn why the pointed arch lets stone float, how a timber centering is struck and a vault suddenly holds itself, and why lime mortar sets the pace of the whole century. Then watch the site put itself to bed, wrapped in straw against the frost, still quietly turning back into stone in the dark.</t>
         </is>
       </c>
       <c r="V12" s="7" t="inlineStr">
@@ -2836,14 +2830,14 @@
       </c>
       <c r="AS12" s="9" t="inlineStr">
         <is>
-          <t>Stories/the-deep-ocean-trenches/story.yaml</t>
+          <t>Stories/the-building-of-a-cathedral/story.yaml</t>
         </is>
       </c>
     </row>
     <row r="13" ht="26" customHeight="1">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>the-great-library-of-alexandria</t>
+          <t>the-clockmaker-s-workshop</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr"/>
@@ -2864,22 +2858,22 @@
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>The Great Library of Alexandria</t>
+          <t>The Clockmaker's Workshop</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>Lamplight, papyrus and patient work beside a warm and quiet sea</t>
+          <t>An evening among a hundred gentle clocks, none of them quite in agreement</t>
         </is>
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>Lullable</t>
         </is>
       </c>
       <c r="I13" s="7" t="inlineStr">
         <is>
-          <t>ancient-worlds</t>
+          <t>cozy-tales</t>
         </is>
       </c>
       <c r="J13" s="7" t="inlineStr"/>
@@ -2900,12 +2894,12 @@
       </c>
       <c r="N13" s="7" t="inlineStr">
         <is>
-          <t>3A2A18</t>
+          <t>1C140E</t>
         </is>
       </c>
       <c r="O13" s="7" t="inlineStr">
         <is>
-          <t>D9A55C</t>
+          <t>C98F3D</t>
         </is>
       </c>
       <c r="P13" s="8" t="inlineStr">
@@ -2915,27 +2909,27 @@
       </c>
       <c r="Q13" s="7" t="inlineStr">
         <is>
-          <t>Nothing here is urgent and nothing needs remembering. Only scribes at their tables, copying one careful line at a time.</t>
+          <t>The shop is locked, the lamp is out, and every pendulum keeps its small agreement in the dark. Nobody has to keep time while they sleep. It is being handled.</t>
         </is>
       </c>
       <c r="R13" s="7" t="inlineStr">
         <is>
-          <t>Slowing a busy day</t>
+          <t>Ticking down to rest</t>
         </is>
       </c>
       <c r="S13" s="7" t="inlineStr">
         <is>
-          <t>Slow, unhurried</t>
+          <t>Once a second, forever</t>
         </is>
       </c>
       <c r="T13" s="7" t="inlineStr">
         <is>
-          <t>Warm, dusty, lamplit</t>
+          <t>Brass, oil, a hundred ticks</t>
         </is>
       </c>
       <c r="U13" s="7" t="inlineStr">
         <is>
-          <t>You arrive at a harbour in the evening, when the light is going gold and the sea wind is moving up through the streets. Inside the cool halls, thousands of scrolls lie in their niches, and scribes copy them by hand, one careful line at a time. You learn how papyrus was pressed from river reeds, how ink was made from soot, how the first catalogue was written, and how a man measured the whole earth from the length of a shadow. Then the lamps are lit, and the work is set down.</t>
+          <t>Step through a door with a brass bell into a small-town shop where a hundred clocks tick softly out of step, like rain on a roof. At the bench, an unhurried craftsman tends a movement of polished wheels with tools that have not changed in two centuries. Learn what a clock really is, a falling weight let down slowly over a week, and why two clocks on the same wall drift into perfect step with each other, a mystery first noticed from a sickbed in 1665. With painted moon dials, a drawer of orphaned keys that all fit something somewhere, winding day, house calls taken over tea, and the repairers' names penciled inside case doors, a century apart.</t>
         </is>
       </c>
       <c r="V13" s="7" t="inlineStr">
@@ -3055,14 +3049,14 @@
       </c>
       <c r="AS13" s="9" t="inlineStr">
         <is>
-          <t>Stories/the-great-library-of-alexandria/story.yaml</t>
+          <t>Stories/the-clockmaker-s-workshop/story.yaml</t>
         </is>
       </c>
     </row>
     <row r="14" ht="26" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>the-joinery-of-japan-s-wooden-temples</t>
+          <t>the-deep-ocean-trenches</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr"/>
@@ -3083,22 +3077,22 @@
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>The Joinery of Japan's Wooden Temples</t>
+          <t>The Deep Ocean Trenches</t>
         </is>
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>Thirteen centuries of buildings held together by shape alone, and not one nail</t>
+          <t>A slow descent past the last of the light, into the stillest water on earth</t>
         </is>
       </c>
       <c r="H14" s="7" t="inlineStr">
         <is>
-          <t>Lullable</t>
+          <t>PENDING</t>
         </is>
       </c>
       <c r="I14" s="7" t="inlineStr">
         <is>
-          <t>ancient-worlds</t>
+          <t>gentle-nature</t>
         </is>
       </c>
       <c r="J14" s="7" t="inlineStr"/>
@@ -3119,12 +3113,12 @@
       </c>
       <c r="N14" s="7" t="inlineStr">
         <is>
-          <t>1E241C</t>
+          <t>0B1F33</t>
         </is>
       </c>
       <c r="O14" s="7" t="inlineStr">
         <is>
-          <t>C4B49A</t>
+          <t>5FA8C4</t>
         </is>
       </c>
       <c r="P14" s="8" t="inlineStr">
@@ -3134,27 +3128,27 @@
       </c>
       <c r="Q14" s="7" t="inlineStr">
         <is>
-          <t>Nothing here was ever nailed, so nothing is ever finished. It has been taken apart and put back together for thirteen hundred years, and none of it needs watching tonight.</t>
+          <t>One slow direction, downward, and nothing waiting at the end of it. An easy thing to follow, and an easier thing to let go of.</t>
         </is>
       </c>
       <c r="R14" s="7" t="inlineStr">
         <is>
-          <t>Putting the day down</t>
+          <t>Letting the day end</t>
         </is>
       </c>
       <c r="S14" s="7" t="inlineStr">
         <is>
-          <t>Careful and unhurried</t>
+          <t>Slow and sinking</t>
         </is>
       </c>
       <c r="T14" s="7" t="inlineStr">
         <is>
-          <t>Wooden, misty, still, warm</t>
+          <t>Dark, cool, weightless</t>
         </is>
       </c>
       <c r="U14" s="7" t="inlineStr">
         <is>
-          <t>Stand in a raked gravel courtyard at dawn and look up at a building with no nails in it. No screws, no brackets, nothing but wood cut to hold wood. Along the way, the joint that grips harder the more you load it, the carpenter who said to buy the mountain rather than the timber, a central pillar that holds up nothing and rests loose on a stone, and roof bark peeled from living trees that grow it back in ten years. And at Ise, a shrine rebuilt from new wood every twenty years for thirteen centuries, because twenty years is the length of human memory.</t>
+          <t>You slip beneath a starlit sea and sink, without effort, through the sunlit water and the long blue twilight into a darkness the sun has never reached. Small living lights blink on and drift away. Marine snow falls, soft and endless, all the way down to a floor of pale sediment older than memory. Further down still lie the trenches, where the pressure feels only like stillness and there is nowhere deeper to go.</t>
         </is>
       </c>
       <c r="V14" s="7" t="inlineStr">
@@ -3274,14 +3268,14 @@
       </c>
       <c r="AS14" s="9" t="inlineStr">
         <is>
-          <t>Stories/the-joinery-of-japan-s-wooden-temples/story.yaml</t>
+          <t>Stories/the-deep-ocean-trenches/story.yaml</t>
         </is>
       </c>
     </row>
     <row r="15" ht="26" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>the-journey-of-a-glacial-river</t>
+          <t>the-great-library-of-alexandria</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr"/>
@@ -3302,22 +3296,22 @@
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>The Journey of a Glacial River</t>
+          <t>The Great Library of Alexandria</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
-          <t>One snowflake's two-hundred-year trip from a silent snowfield to the sea</t>
+          <t>Lamplight, papyrus and patient work beside a warm and quiet sea</t>
         </is>
       </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>Lullable</t>
+          <t>PENDING</t>
         </is>
       </c>
       <c r="I15" s="7" t="inlineStr">
         <is>
-          <t>gentle-nature</t>
+          <t>ancient-worlds</t>
         </is>
       </c>
       <c r="J15" s="7" t="inlineStr"/>
@@ -3338,12 +3332,12 @@
       </c>
       <c r="N15" s="7" t="inlineStr">
         <is>
-          <t>0F2230</t>
+          <t>3A2A18</t>
         </is>
       </c>
       <c r="O15" s="7" t="inlineStr">
         <is>
-          <t>7FD0C9</t>
+          <t>D9A55C</t>
         </is>
       </c>
       <c r="P15" s="8" t="inlineStr">
@@ -3353,27 +3347,27 @@
       </c>
       <c r="Q15" s="7" t="inlineStr">
         <is>
-          <t>Water never has to choose. It goes the one way it can go, at whatever pace it is given, and tonight you can go with it, downhill the whole way.</t>
+          <t>Nothing here is urgent and nothing needs remembering. Only scribes at their tables, copying one careful line at a time.</t>
         </is>
       </c>
       <c r="R15" s="7" t="inlineStr">
         <is>
-          <t>Drifting downstream</t>
+          <t>Slowing a busy day</t>
         </is>
       </c>
       <c r="S15" s="7" t="inlineStr">
         <is>
-          <t>Downhill, all the way</t>
+          <t>Slow, unhurried</t>
         </is>
       </c>
       <c r="T15" s="7" t="inlineStr">
         <is>
-          <t>Blue ice, cold water, calm</t>
+          <t>Warm, dusty, lamplit</t>
         </is>
       </c>
       <c r="U15" s="7" t="inlineStr">
         <is>
-          <t>Follow a single snowflake from a windless high snowfield down to the salt water, a journey of two centuries in one direction only. Be buried into blue glacier ice with a breath of old sky sealed inside, ride the slowest river there is, and emerge at the ice cave where the young river is born, milky with the flour of ground mountains. Then down through the braided gravel plains, into a turquoise lake that sorts the sunlight, through pine forests where a small brown bird walks underwater, and out at last across the mudflats to the sea, where the sun is already lifting the water to begin again.</t>
+          <t>You arrive at a harbour in the evening, when the light is going gold and the sea wind is moving up through the streets. Inside the cool halls, thousands of scrolls lie in their niches, and scribes copy them by hand, one careful line at a time. You learn how papyrus was pressed from river reeds, how ink was made from soot, how the first catalogue was written, and how a man measured the whole earth from the length of a shadow. Then the lamps are lit, and the work is set down.</t>
         </is>
       </c>
       <c r="V15" s="7" t="inlineStr">
@@ -3493,14 +3487,14 @@
       </c>
       <c r="AS15" s="9" t="inlineStr">
         <is>
-          <t>Stories/the-journey-of-a-glacial-river/story.yaml</t>
+          <t>Stories/the-great-library-of-alexandria/story.yaml</t>
         </is>
       </c>
     </row>
     <row r="16" ht="26" customHeight="1">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>the-life-cycle-of-a-red-dwarf-star</t>
+          <t>the-joinery-of-japan-s-wooden-temples</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr"/>
@@ -3521,12 +3515,12 @@
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>The Life Cycle of a Red Dwarf Star</t>
+          <t>The Joinery of Japan's Wooden Temples</t>
         </is>
       </c>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>The commonest star in the galaxy, burning so slowly that none has ever finished</t>
+          <t>Thirteen centuries of buildings held together by shape alone, and not one nail</t>
         </is>
       </c>
       <c r="H16" s="7" t="inlineStr">
@@ -3536,7 +3530,7 @@
       </c>
       <c r="I16" s="7" t="inlineStr">
         <is>
-          <t>cosmic-journeys</t>
+          <t>ancient-worlds</t>
         </is>
       </c>
       <c r="J16" s="7" t="inlineStr"/>
@@ -3557,12 +3551,12 @@
       </c>
       <c r="N16" s="7" t="inlineStr">
         <is>
-          <t>1C1013</t>
+          <t>1E241C</t>
         </is>
       </c>
       <c r="O16" s="7" t="inlineStr">
         <is>
-          <t>D97A55</t>
+          <t>C4B49A</t>
         </is>
       </c>
       <c r="P16" s="8" t="inlineStr">
@@ -3572,27 +3566,27 @@
       </c>
       <c r="Q16" s="7" t="inlineStr">
         <is>
-          <t>Not one red dwarf has ever run down. The universe is far too young. Every single one ever made is still quietly burning, and none of it needs watching tonight.</t>
+          <t>Nothing here was ever nailed, so nothing is ever finished. It has been taken apart and put back together for thirteen hundred years, and none of it needs watching tonight.</t>
         </is>
       </c>
       <c r="R16" s="7" t="inlineStr">
         <is>
-          <t>Unwinding without hurry</t>
+          <t>Putting the day down</t>
         </is>
       </c>
       <c r="S16" s="7" t="inlineStr">
         <is>
-          <t>Low, warm, unchanging</t>
+          <t>Careful and unhurried</t>
         </is>
       </c>
       <c r="T16" s="7" t="inlineStr">
         <is>
-          <t>Dim, orange, warm, endless</t>
+          <t>Wooden, misty, still, warm</t>
         </is>
       </c>
       <c r="U16" s="7" t="inlineStr">
         <is>
-          <t>Travel four light years to Proxima Centauri, a small orange star so dim you could look straight at it, and so ordinary that three quarters of the galaxy is made of stars like it. Inside, the whole body slowly turns itself over, which is why it will still be burning in ten trillion years. Along the way, why nature makes far more small stars than large ones, the women at Harvard who sorted the spectra by hand, the titanium chemistry that survives in a star's atmosphere, and the quiet fact that not one red dwarf anywhere has ever finished.</t>
+          <t>Stand in a raked gravel courtyard at dawn and look up at a building with no nails in it. No screws, no brackets, nothing but wood cut to hold wood. Along the way, the joint that grips harder the more you load it, the carpenter who said to buy the mountain rather than the timber, a central pillar that holds up nothing and rests loose on a stone, and roof bark peeled from living trees that grow it back in ten years. And at Ise, a shrine rebuilt from new wood every twenty years for thirteen centuries, because twenty years is the length of human memory.</t>
         </is>
       </c>
       <c r="V16" s="7" t="inlineStr">
@@ -3712,14 +3706,14 @@
       </c>
       <c r="AS16" s="9" t="inlineStr">
         <is>
-          <t>Stories/the-life-cycle-of-a-red-dwarf-star/story.yaml</t>
+          <t>Stories/the-joinery-of-japan-s-wooden-temples/story.yaml</t>
         </is>
       </c>
     </row>
     <row r="17" ht="26" customHeight="1">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>the-midnight-sleeper-train-across-the-alps</t>
+          <t>the-journey-of-a-glacial-river</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr"/>
@@ -3740,12 +3734,12 @@
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>The Midnight Sleeper Train Across the Alps</t>
+          <t>The Journey of a Glacial River</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>A warm berth, a folder of sleeping passports, and mountains passing in the dark</t>
+          <t>One snowflake's two-hundred-year trip from a silent snowfield to the sea</t>
         </is>
       </c>
       <c r="H17" s="7" t="inlineStr">
@@ -3755,7 +3749,7 @@
       </c>
       <c r="I17" s="7" t="inlineStr">
         <is>
-          <t>cozy-tales</t>
+          <t>gentle-nature</t>
         </is>
       </c>
       <c r="J17" s="7" t="inlineStr"/>
@@ -3776,12 +3770,12 @@
       </c>
       <c r="N17" s="7" t="inlineStr">
         <is>
-          <t>151A2E</t>
+          <t>0F2230</t>
         </is>
       </c>
       <c r="O17" s="7" t="inlineStr">
         <is>
-          <t>D9B36C</t>
+          <t>7FD0C9</t>
         </is>
       </c>
       <c r="P17" s="8" t="inlineStr">
@@ -3791,27 +3785,27 @@
       </c>
       <c r="Q17" s="7" t="inlineStr">
         <is>
-          <t>The signals are turning green all the way to the lake, and the attendant is awake so you need not be. The train knows the rest, and none of it is your business tonight.</t>
+          <t>Water never has to choose. It goes the one way it can go, at whatever pace it is given, and tonight you can go with it, downhill the whole way.</t>
         </is>
       </c>
       <c r="R17" s="7" t="inlineStr">
         <is>
-          <t>Being gently carried</t>
+          <t>Drifting downstream</t>
         </is>
       </c>
       <c r="S17" s="7" t="inlineStr">
         <is>
-          <t>Rocking and westward</t>
+          <t>Downhill, all the way</t>
         </is>
       </c>
       <c r="T17" s="7" t="inlineStr">
         <is>
-          <t>Warm, amber, moonlit, moving</t>
+          <t>Blue ice, cold water, calm</t>
         </is>
       </c>
       <c r="U17" s="7" t="inlineStr">
         <is>
-          <t>Board the midnight-blue sleeper in Vienna, hand your passport to the attendant, and let the train do the rest. Cross the Alps in a rocking berth while borders pass over you like weather, carriages are quietly sorted toward separate mornings, and a freight train washes past in the dark. Along the way, why the clickety-clack disappeared when the rails were welded into seamless miles, the 1884 tunnel bored from both ends to meet like a handshake, and the whole quiet profession of people who stay awake so that everyone else can sleep at seventy miles an hour.</t>
+          <t>Follow a single snowflake from a windless high snowfield down to the salt water, a journey of two centuries in one direction only. Be buried into blue glacier ice with a breath of old sky sealed inside, ride the slowest river there is, and emerge at the ice cave where the young river is born, milky with the flour of ground mountains. Then down through the braided gravel plains, into a turquoise lake that sorts the sunlight, through pine forests where a small brown bird walks underwater, and out at last across the mudflats to the sea, where the sun is already lifting the water to begin again.</t>
         </is>
       </c>
       <c r="V17" s="7" t="inlineStr">
@@ -3931,14 +3925,14 @@
       </c>
       <c r="AS17" s="9" t="inlineStr">
         <is>
-          <t>Stories/the-midnight-sleeper-train-across-the-alps/story.yaml</t>
+          <t>Stories/the-journey-of-a-glacial-river/story.yaml</t>
         </is>
       </c>
     </row>
     <row r="18" ht="26" customHeight="1">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>the-moons-of-jupiter-europa-s-ice-and-ocean</t>
+          <t>the-life-cycle-of-a-red-dwarf-star</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr"/>
@@ -3959,12 +3953,12 @@
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
-          <t>The Moons of Jupiter: Europa's Ice and Ocean</t>
+          <t>The Life Cycle of a Red Dwarf Star</t>
         </is>
       </c>
       <c r="G18" s="7" t="inlineStr">
         <is>
-          <t>A small cracked moon of ice, and the dark ocean turning over beneath it</t>
+          <t>The commonest star in the galaxy, burning so slowly that none has ever finished</t>
         </is>
       </c>
       <c r="H18" s="7" t="inlineStr">
@@ -3995,12 +3989,12 @@
       </c>
       <c r="N18" s="7" t="inlineStr">
         <is>
-          <t>0E1A2B</t>
+          <t>1C1013</t>
         </is>
       </c>
       <c r="O18" s="7" t="inlineStr">
         <is>
-          <t>9FC8DA</t>
+          <t>D97A55</t>
         </is>
       </c>
       <c r="P18" s="8" t="inlineStr">
@@ -4010,27 +4004,27 @@
       </c>
       <c r="Q18" s="7" t="inlineStr">
         <is>
-          <t>There is no light down there and there never has been. The water simply turns over in the dark, as it has for a very long time, and none of it needs watching tonight.</t>
+          <t>Not one red dwarf has ever run down. The universe is far too young. Every single one ever made is still quietly burning, and none of it needs watching tonight.</t>
         </is>
       </c>
       <c r="R18" s="7" t="inlineStr">
         <is>
-          <t>Sinking into sleep</t>
+          <t>Unwinding without hurry</t>
         </is>
       </c>
       <c r="S18" s="7" t="inlineStr">
         <is>
-          <t>Quiet and downward</t>
+          <t>Low, warm, unchanging</t>
         </is>
       </c>
       <c r="T18" s="7" t="inlineStr">
         <is>
-          <t>Cold, white, deep, quiet</t>
+          <t>Dim, orange, warm, endless</t>
         </is>
       </c>
       <c r="U18" s="7" t="inlineStr">
         <is>
-          <t>You travel out past Mars to a banded planet eleven times the width of the Earth, and find four small worlds standing beside it in a line. The second one is white, smooth as a billiard ball, and cracked all over like a glazed bowl. You learn why it has almost no craters, how a tiny wobble in its orbit keeps an ocean liquid where nothing should be, and how that ocean was found from the outside without anyone touching it. Then you sink through the ice into water that has never once seen light.</t>
+          <t>Travel four light years to Proxima Centauri, a small orange star so dim you could look straight at it, and so ordinary that three quarters of the galaxy is made of stars like it. Inside, the whole body slowly turns itself over, which is why it will still be burning in ten trillion years. Along the way, why nature makes far more small stars than large ones, the women at Harvard who sorted the spectra by hand, the titanium chemistry that survives in a star's atmosphere, and the quiet fact that not one red dwarf anywhere has ever finished.</t>
         </is>
       </c>
       <c r="V18" s="7" t="inlineStr">
@@ -4150,14 +4144,14 @@
       </c>
       <c r="AS18" s="9" t="inlineStr">
         <is>
-          <t>Stories/the-moons-of-jupiter-europa-s-ice-and-ocean/story.yaml</t>
+          <t>Stories/the-life-cycle-of-a-red-dwarf-star/story.yaml</t>
         </is>
       </c>
     </row>
     <row r="19" ht="26" customHeight="1">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>the-observatory-on-ben-nevis</t>
+          <t>the-midnight-sleeper-train-across-the-alps</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr"/>
@@ -4178,17 +4172,17 @@
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>The Observatory on Ben Nevis</t>
+          <t>The Midnight Sleeper Train Across the Alps</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>Twenty-one years of hourly weather readings, taken by lamplight inside a cloud</t>
+          <t>A warm berth, a folder of sleeping passports, and mountains passing in the dark</t>
         </is>
       </c>
       <c r="H19" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>Lullable</t>
         </is>
       </c>
       <c r="I19" s="7" t="inlineStr">
@@ -4214,12 +4208,12 @@
       </c>
       <c r="N19" s="7" t="inlineStr">
         <is>
-          <t>1F2A2E</t>
+          <t>151A2E</t>
         </is>
       </c>
       <c r="O19" s="7" t="inlineStr">
         <is>
-          <t>B9C9CE</t>
+          <t>D9B36C</t>
         </is>
       </c>
       <c r="P19" s="8" t="inlineStr">
@@ -4229,27 +4223,27 @@
       </c>
       <c r="Q19" s="7" t="inlineStr">
         <is>
-          <t>Somebody is awake on a mountain, taking a reading on the hour, whether or not you are. The next one is not yours, and it will be taken anyway.</t>
+          <t>The signals are turning green all the way to the lake, and the attendant is awake so you need not be. The train knows the rest, and none of it is your business tonight.</t>
         </is>
       </c>
       <c r="R19" s="7" t="inlineStr">
         <is>
-          <t>Letting go of the day</t>
+          <t>Being gently carried</t>
         </is>
       </c>
       <c r="S19" s="7" t="inlineStr">
         <is>
-          <t>Hourly and unhurried</t>
+          <t>Rocking and westward</t>
         </is>
       </c>
       <c r="T19" s="7" t="inlineStr">
         <is>
-          <t>Cold, lamplit, patient</t>
+          <t>Warm, amber, moonlit, moving</t>
         </is>
       </c>
       <c r="U19" s="7" t="inlineStr">
         <is>
-          <t>You climb into the cloud that sits on the highest ground in Britain, and step through a low stone door into lamplight, a warm stove, and a kettle that is always on. For twenty-one years, somebody here walked out into the weather every hour of every night and wrote down what it was doing. You learn how a wet sleeve of muslin measures the dryness of the air, why the thermometer boxes had to be lifted as the snow came up to meet them, and how ice grows sideways into the wind. Then the lamp is turned low, a wet coat goes on the hook, and the mountain carries on without you.</t>
+          <t>Board the midnight-blue sleeper in Vienna, hand your passport to the attendant, and let the train do the rest. Cross the Alps in a rocking berth while borders pass over you like weather, carriages are quietly sorted toward separate mornings, and a freight train washes past in the dark. Along the way, why the clickety-clack disappeared when the rails were welded into seamless miles, the 1884 tunnel bored from both ends to meet like a handshake, and the whole quiet profession of people who stay awake so that everyone else can sleep at seventy miles an hour.</t>
         </is>
       </c>
       <c r="V19" s="7" t="inlineStr">
@@ -4369,40 +4363,40 @@
       </c>
       <c r="AS19" s="9" t="inlineStr">
         <is>
-          <t>Stories/the-observatory-on-ben-nevis/story.yaml</t>
+          <t>Stories/the-midnight-sleeper-train-across-the-alps/story.yaml</t>
         </is>
       </c>
     </row>
     <row r="20" ht="26" customHeight="1">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>the-rings-of-saturn</t>
+          <t>the-moons-of-jupiter-europa-s-ice-and-ocean</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr"/>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>published</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>free</t>
+          <t>premium</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>free</t>
+          <t>PENDING</t>
         </is>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>The Rings of Saturn</t>
+          <t>The Moons of Jupiter: Europa's Ice and Ocean</t>
         </is>
       </c>
       <c r="G20" s="7" t="inlineStr">
         <is>
-          <t>Ten metres of ice, two hundred thousand kilometres wide, turning in silence</t>
+          <t>A small cracked moon of ice, and the dark ocean turning over beneath it</t>
         </is>
       </c>
       <c r="H20" s="7" t="inlineStr">
@@ -4423,60 +4417,62 @@
       </c>
       <c r="L20" s="7" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>false</t>
         </is>
       </c>
       <c r="M20" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14T17:53:16Z</t>
+          <t>PENDING</t>
         </is>
       </c>
       <c r="N20" s="7" t="inlineStr">
         <is>
-          <t>1B2436</t>
+          <t>0E1A2B</t>
         </is>
       </c>
       <c r="O20" s="7" t="inlineStr">
         <is>
-          <t>E8C89A</t>
-        </is>
-      </c>
-      <c r="P20" s="8" t="n">
-        <v>2125.557</v>
+          <t>9FC8DA</t>
+        </is>
+      </c>
+      <c r="P20" s="8" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
       </c>
       <c r="Q20" s="7" t="inlineStr">
         <is>
-          <t>A long way from anything that has ever asked something of you. Nothing out here is in a hurry, and none of it needs watching.</t>
+          <t>There is no light down there and there never has been. The water simply turns over in the dark, as it has for a very long time, and none of it needs watching tonight.</t>
         </is>
       </c>
       <c r="R20" s="7" t="inlineStr">
         <is>
-          <t>Drifting off slowly</t>
+          <t>Sinking into sleep</t>
         </is>
       </c>
       <c r="S20" s="7" t="inlineStr">
         <is>
-          <t>Slow and weightless</t>
+          <t>Quiet and downward</t>
         </is>
       </c>
       <c r="T20" s="7" t="inlineStr">
         <is>
-          <t>Cold, vast, silent</t>
+          <t>Cold, white, deep, quiet</t>
         </is>
       </c>
       <c r="U20" s="7" t="inlineStr">
         <is>
-          <t>You rise gently from your own roof and travel outward, past the Moon and Jupiter, until a tilted gold shape appears in the dark. Up close the rings resolve into thousands of fine bright lines, and then into ice: billions of frozen pieces, some finer than dust and some the size of mountains, all drifting the same way at once. You watch small moons carve clean lanes and raise slow waves behind them, hear a gentle unfinished argument about how old it all is, and then settle into the ring plane and stay.</t>
+          <t>You travel out past Mars to a banded planet eleven times the width of the Earth, and find four small worlds standing beside it in a line. The second one is white, smooth as a billiard ball, and cracked all over like a glazed bowl. You learn why it has almost no craters, how a tiny wobble in its orbit keeps an ocean liquid where nothing should be, and how that ocean was found from the outside without anyone touching it. Then you sink through the ice into water that has never once seen light.</t>
         </is>
       </c>
       <c r="V20" s="7" t="inlineStr">
         <is>
-          <t>audio-the-rings-of-saturn-en-v2-aac96</t>
+          <t>PENDING</t>
         </is>
       </c>
       <c r="W20" s="7" t="inlineStr">
         <is>
-          <t>ElevenLabs_the-rings-of-saturn-v2.wav</t>
+          <t>PENDING</t>
         </is>
       </c>
       <c r="X20" s="7" t="inlineStr">
@@ -4491,12 +4487,12 @@
       </c>
       <c r="Z20" s="9" t="inlineStr">
         <is>
-          <t>published</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="AA20" s="9" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>NOT READY</t>
         </is>
       </c>
       <c r="AB20" s="9" t="inlineStr">
@@ -4526,47 +4522,47 @@
       </c>
       <c r="AG20" s="9" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="AH20" s="9" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="AI20" s="9" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="AJ20" s="9" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="AK20" s="9" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="AL20" s="9" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="AM20" s="9" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="AN20" s="9" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="AO20" s="9" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="AP20" s="9" t="inlineStr">
@@ -4586,14 +4582,14 @@
       </c>
       <c r="AS20" s="9" t="inlineStr">
         <is>
-          <t>Stories/the-rings-of-saturn/story.yaml</t>
+          <t>Stories/the-moons-of-jupiter-europa-s-ice-and-ocean/story.yaml</t>
         </is>
       </c>
     </row>
     <row r="21" ht="26" customHeight="1">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>the-slow-life-of-a-redwood</t>
+          <t>the-observatory-on-ben-nevis</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr"/>
@@ -4614,22 +4610,22 @@
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>The Slow Life of a Redwood</t>
+          <t>The Observatory on Ben Nevis</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
         <is>
-          <t>A night in the fog with the tallest living things there have ever been</t>
+          <t>Twenty-one years of hourly weather readings, taken by lamplight inside a cloud</t>
         </is>
       </c>
       <c r="H21" s="7" t="inlineStr">
         <is>
-          <t>Lullable</t>
+          <t>PENDING</t>
         </is>
       </c>
       <c r="I21" s="7" t="inlineStr">
         <is>
-          <t>gentle-nature</t>
+          <t>cozy-tales</t>
         </is>
       </c>
       <c r="J21" s="7" t="inlineStr"/>
@@ -4650,12 +4646,12 @@
       </c>
       <c r="N21" s="7" t="inlineStr">
         <is>
-          <t>14201A</t>
+          <t>1F2A2E</t>
         </is>
       </c>
       <c r="O21" s="7" t="inlineStr">
         <is>
-          <t>A8C3A0</t>
+          <t>B9C9CE</t>
         </is>
       </c>
       <c r="P21" s="8" t="inlineStr">
@@ -4665,27 +4661,27 @@
       </c>
       <c r="Q21" s="7" t="inlineStr">
         <is>
-          <t>The grove waters itself with fog while everyone sleeps, and has done for two thousand summers. Nothing in it moves faster than a slug, and nothing needs watching tonight.</t>
+          <t>Somebody is awake on a mountain, taking a reading on the hour, whether or not you are. The next one is not yours, and it will be taken anyway.</t>
         </is>
       </c>
       <c r="R21" s="7" t="inlineStr">
         <is>
-          <t>Quieting a full mind</t>
+          <t>Letting go of the day</t>
         </is>
       </c>
       <c r="S21" s="7" t="inlineStr">
         <is>
-          <t>Soft, green, ancient</t>
+          <t>Hourly and unhurried</t>
         </is>
       </c>
       <c r="T21" s="7" t="inlineStr">
         <is>
-          <t>Foggy, hushed, deep green</t>
+          <t>Cold, lamplit, patient</t>
         </is>
       </c>
       <c r="U21" s="7" t="inlineStr">
         <is>
-          <t>Walk into a coastal grove at dusk and stand at the foot of a tree over three hundred feet tall, wrapped in a foot of soft bark, older than the cathedrals. Follow one unbroken thread of water from the roots to the highest needle, and wait for the summer fog to roll in off the cold Pacific so the forest can water itself in the dark. Along the way, roots that graft into their neighbours and hold each other up, rings of trees standing where their elders stood, a ghost-white redwood fed by its family, and a garden of ferns and huckleberries growing a metre deep in the crown.</t>
+          <t>You climb into the cloud that sits on the highest ground in Britain, and step through a low stone door into lamplight, a warm stove, and a kettle that is always on. For twenty-one years, somebody here walked out into the weather every hour of every night and wrote down what it was doing. You learn how a wet sleeve of muslin measures the dryness of the air, why the thermometer boxes had to be lifted as the snow came up to meet them, and how ice grows sideways into the wind. Then the lamp is turned low, a wet coat goes on the hook, and the mountain carries on without you.</t>
         </is>
       </c>
       <c r="V21" s="7" t="inlineStr">
@@ -4805,40 +4801,40 @@
       </c>
       <c r="AS21" s="9" t="inlineStr">
         <is>
-          <t>Stories/the-slow-life-of-a-redwood/story.yaml</t>
+          <t>Stories/the-observatory-on-ben-nevis/story.yaml</t>
         </is>
       </c>
     </row>
     <row r="22" ht="26" customHeight="1">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>voyager-1-a-journey-to-interstellar-space</t>
+          <t>the-rings-of-saturn</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr"/>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>published</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>premium</t>
+          <t>free</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>free</t>
         </is>
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
-          <t>Voyager 1: A Journey to Interstellar Space</t>
+          <t>The Rings of Saturn</t>
         </is>
       </c>
       <c r="G22" s="7" t="inlineStr">
         <is>
-          <t>A small gold machine, forty-nine years out, still quietly drifting away from us</t>
+          <t>Ten metres of ice, two hundred thousand kilometres wide, turning in silence</t>
         </is>
       </c>
       <c r="H22" s="7" t="inlineStr">
@@ -4859,177 +4855,613 @@
       </c>
       <c r="L22" s="7" t="inlineStr">
         <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="M22" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-14T17:53:16Z</t>
+        </is>
+      </c>
+      <c r="N22" s="7" t="inlineStr">
+        <is>
+          <t>1B2436</t>
+        </is>
+      </c>
+      <c r="O22" s="7" t="inlineStr">
+        <is>
+          <t>E8C89A</t>
+        </is>
+      </c>
+      <c r="P22" s="8" t="n">
+        <v>2125.557</v>
+      </c>
+      <c r="Q22" s="7" t="inlineStr">
+        <is>
+          <t>A long way from anything that has ever asked something of you. Nothing out here is in a hurry, and none of it needs watching.</t>
+        </is>
+      </c>
+      <c r="R22" s="7" t="inlineStr">
+        <is>
+          <t>Drifting off slowly</t>
+        </is>
+      </c>
+      <c r="S22" s="7" t="inlineStr">
+        <is>
+          <t>Slow and weightless</t>
+        </is>
+      </c>
+      <c r="T22" s="7" t="inlineStr">
+        <is>
+          <t>Cold, vast, silent</t>
+        </is>
+      </c>
+      <c r="U22" s="7" t="inlineStr">
+        <is>
+          <t>You rise gently from your own roof and travel outward, past the Moon and Jupiter, until a tilted gold shape appears in the dark. Up close the rings resolve into thousands of fine bright lines, and then into ice: billions of frozen pieces, some finer than dust and some the size of mountains, all drifting the same way at once. You watch small moons carve clean lanes and raise slow waves behind them, hear a gentle unfinished argument about how old it all is, and then settle into the ring plane and stay.</t>
+        </is>
+      </c>
+      <c r="V22" s="7" t="inlineStr">
+        <is>
+          <t>audio-the-rings-of-saturn-en-v2-aac96</t>
+        </is>
+      </c>
+      <c r="W22" s="7" t="inlineStr">
+        <is>
+          <t>ElevenLabs_the-rings-of-saturn-v2.wav</t>
+        </is>
+      </c>
+      <c r="X22" s="7" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="Y22" s="7" t="inlineStr">
+        <is>
+          <t>AAC-LC M4A, 44.1 kHz, mono, 96 kbps</t>
+        </is>
+      </c>
+      <c r="Z22" s="9" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="AA22" s="9" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="AB22" s="9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AC22" s="9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AD22" s="9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AE22" s="9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AF22" s="9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AG22" s="9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AH22" s="9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AI22" s="9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AJ22" s="9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AK22" s="9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AL22" s="9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AM22" s="9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AN22" s="9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AO22" s="9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AP22" s="9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AQ22" s="9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AR22" s="9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AS22" s="9" t="inlineStr">
+        <is>
+          <t>Stories/the-rings-of-saturn/story.yaml</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="26" customHeight="1">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>the-slow-life-of-a-redwood</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr"/>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>premium</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>The Slow Life of a Redwood</t>
+        </is>
+      </c>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>A night in the fog with the tallest living things there have ever been</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>Lullable</t>
+        </is>
+      </c>
+      <c r="I23" s="7" t="inlineStr">
+        <is>
+          <t>gentle-nature</t>
+        </is>
+      </c>
+      <c r="J23" s="7" t="inlineStr"/>
+      <c r="K23" s="7" t="inlineStr">
+        <is>
           <t>false</t>
         </is>
       </c>
-      <c r="M22" s="7" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="N22" s="7" t="inlineStr">
+      <c r="L23" s="7" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="M23" s="7" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="N23" s="7" t="inlineStr">
+        <is>
+          <t>14201A</t>
+        </is>
+      </c>
+      <c r="O23" s="7" t="inlineStr">
+        <is>
+          <t>A8C3A0</t>
+        </is>
+      </c>
+      <c r="P23" s="8" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="Q23" s="7" t="inlineStr">
+        <is>
+          <t>The grove waters itself with fog while everyone sleeps, and has done for two thousand summers. Nothing in it moves faster than a slug, and nothing needs watching tonight.</t>
+        </is>
+      </c>
+      <c r="R23" s="7" t="inlineStr">
+        <is>
+          <t>Quieting a full mind</t>
+        </is>
+      </c>
+      <c r="S23" s="7" t="inlineStr">
+        <is>
+          <t>Soft, green, ancient</t>
+        </is>
+      </c>
+      <c r="T23" s="7" t="inlineStr">
+        <is>
+          <t>Foggy, hushed, deep green</t>
+        </is>
+      </c>
+      <c r="U23" s="7" t="inlineStr">
+        <is>
+          <t>Walk into a coastal grove at dusk and stand at the foot of a tree over three hundred feet tall, wrapped in a foot of soft bark, older than the cathedrals. Follow one unbroken thread of water from the roots to the highest needle, and wait for the summer fog to roll in off the cold Pacific so the forest can water itself in the dark. Along the way, roots that graft into their neighbours and hold each other up, rings of trees standing where their elders stood, a ghost-white redwood fed by its family, and a garden of ferns and huckleberries growing a metre deep in the crown.</t>
+        </is>
+      </c>
+      <c r="V23" s="7" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="W23" s="7" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="X23" s="7" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="Y23" s="7" t="inlineStr">
+        <is>
+          <t>AAC-LC M4A, 44.1 kHz, mono, 96 kbps</t>
+        </is>
+      </c>
+      <c r="Z23" s="9" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="AA23" s="9" t="inlineStr">
+        <is>
+          <t>NOT READY</t>
+        </is>
+      </c>
+      <c r="AB23" s="9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AC23" s="9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AD23" s="9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AE23" s="9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AF23" s="9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AG23" s="9" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="AH23" s="9" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="AI23" s="9" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="AJ23" s="9" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="AK23" s="9" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="AL23" s="9" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="AM23" s="9" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="AN23" s="9" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="AO23" s="9" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="AP23" s="9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AQ23" s="9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AR23" s="9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AS23" s="9" t="inlineStr">
+        <is>
+          <t>Stories/the-slow-life-of-a-redwood/story.yaml</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="26" customHeight="1">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>voyager-1-a-journey-to-interstellar-space</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr"/>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>premium</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>Voyager 1: A Journey to Interstellar Space</t>
+        </is>
+      </c>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>A small gold machine, forty-nine years out, still quietly drifting away from us</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>Lullable</t>
+        </is>
+      </c>
+      <c r="I24" s="7" t="inlineStr">
+        <is>
+          <t>cosmic-journeys</t>
+        </is>
+      </c>
+      <c r="J24" s="7" t="inlineStr"/>
+      <c r="K24" s="7" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="L24" s="7" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="M24" s="7" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="N24" s="7" t="inlineStr">
         <is>
           <t>0A0F1C</t>
         </is>
       </c>
-      <c r="O22" s="7" t="inlineStr">
+      <c r="O24" s="7" t="inlineStr">
         <is>
           <t>C7B27A</t>
         </is>
       </c>
-      <c r="P22" s="8" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="Q22" s="7" t="inlineStr">
+      <c r="P24" s="8" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="Q24" s="7" t="inlineStr">
         <is>
           <t>It left in 1977 and it is not going anywhere in particular. It is simply still going, steadily, and none of it needs watching tonight.</t>
         </is>
       </c>
-      <c r="R22" s="7" t="inlineStr">
+      <c r="R24" s="7" t="inlineStr">
         <is>
           <t>Settling into the quiet</t>
         </is>
       </c>
-      <c r="S22" s="7" t="inlineStr">
+      <c r="S24" s="7" t="inlineStr">
         <is>
           <t>Steady and outward</t>
         </is>
       </c>
-      <c r="T22" s="7" t="inlineStr">
+      <c r="T24" s="7" t="inlineStr">
         <is>
           <t>Dark, distant, gold, calm</t>
         </is>
       </c>
-      <c r="U22" s="7" t="inlineStr">
+      <c r="U24" s="7" t="inlineStr">
         <is>
           <t>Follow the most distant object people have ever made, out past Jupiter and Saturn and into the space between the stars. A gold record bolted to its side, a transmitter no brighter than a refrigerator bulb, and a whisper of radio that takes almost a full day to reach a dish in the Australian grass. Along the way, the gentle theft of a gravity assist, the choice to look at Titan, and the faint steady hum the gas out there turns out to make. Nothing about it is urgent. Nothing about it ever was.</t>
         </is>
       </c>
-      <c r="V22" s="7" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="W22" s="7" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="X22" s="7" t="inlineStr">
+      <c r="V24" s="7" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="W24" s="7" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="X24" s="7" t="inlineStr">
         <is>
           <t>verified</t>
         </is>
       </c>
-      <c r="Y22" s="7" t="inlineStr">
+      <c r="Y24" s="7" t="inlineStr">
         <is>
           <t>AAC-LC M4A, 44.1 kHz, mono, 96 kbps</t>
         </is>
       </c>
-      <c r="Z22" s="9" t="inlineStr">
+      <c r="Z24" s="9" t="inlineStr">
         <is>
           <t>draft</t>
         </is>
       </c>
-      <c r="AA22" s="9" t="inlineStr">
+      <c r="AA24" s="9" t="inlineStr">
         <is>
           <t>NOT READY</t>
         </is>
       </c>
-      <c r="AB22" s="9" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="AC22" s="9" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="AD22" s="9" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="AE22" s="9" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="AF22" s="9" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="AG22" s="9" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="AH22" s="9" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="AI22" s="9" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="AJ22" s="9" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="AK22" s="9" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="AL22" s="9" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="AM22" s="9" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="AN22" s="9" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="AO22" s="9" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="AP22" s="9" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="AQ22" s="9" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="AR22" s="9" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="AS22" s="9" t="inlineStr">
+      <c r="AB24" s="9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AC24" s="9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AD24" s="9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AE24" s="9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AF24" s="9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AG24" s="9" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="AH24" s="9" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="AI24" s="9" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="AJ24" s="9" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="AK24" s="9" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="AL24" s="9" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="AM24" s="9" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="AN24" s="9" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="AO24" s="9" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="AP24" s="9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AQ24" s="9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AR24" s="9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AS24" s="9" t="inlineStr">
         <is>
           <t>Stories/voyager-1-a-journey-to-interstellar-space/story.yaml</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:AS22"/>
+  <autoFilter ref="A3:AS24"/>
   <mergeCells count="6">
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="A2:B2"/>
@@ -5038,7 +5470,7 @@
     <mergeCell ref="A1:AS1"/>
     <mergeCell ref="F2:Y2"/>
   </mergeCells>
-  <conditionalFormatting sqref="AB5:AS22">
+  <conditionalFormatting sqref="AB5:AS24">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"FAIL"</formula>
     </cfRule>
@@ -5046,7 +5478,7 @@
       <formula>"PASS"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AA5:AA22">
+  <conditionalFormatting sqref="AA5:AA24">
     <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
       <formula>"READY"</formula>
     </cfRule>
@@ -5054,31 +5486,31 @@
       <formula>"NOT READY"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D5:D22">
+  <conditionalFormatting sqref="D5:D24">
     <cfRule type="cellIs" priority="5" operator="equal" dxfId="3">
       <formula>"PENDING"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="7">
-    <dataValidation sqref="C5:C62" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Rejected" error="Not an allowed value. Pick from the list." promptTitle="workflowStatus" prompt="Pipeline stage." type="list" errorStyle="stop">
+    <dataValidation sqref="C5:C64" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Rejected" error="Not an allowed value. Pick from the list." promptTitle="workflowStatus" prompt="Pipeline stage." type="list" errorStyle="stop">
       <formula1>"draft,rendered,qa-approved,staging,published"</formula1>
     </dataValidation>
-    <dataValidation sqref="D5:D62" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Rejected" error="Not an allowed value. Pick from the list." promptTitle="accessDecision" prompt="Free vs premium. Settle before staging." type="list" errorStyle="stop">
+    <dataValidation sqref="D5:D64" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Rejected" error="Not an allowed value. Pick from the list." promptTitle="accessDecision" prompt="Free vs premium. Settle before staging." type="list" errorStyle="stop">
       <formula1>"PENDING,free,premium"</formula1>
     </dataValidation>
-    <dataValidation sqref="I5:I62" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Rejected" error="Not an allowed value. Pick from the list." promptTitle="genreID_1" prompt="Existing genre IDs only." type="list" errorStyle="stop">
+    <dataValidation sqref="I5:I64" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Rejected" error="Not an allowed value. Pick from the list." promptTitle="genreID_1" prompt="Existing genre IDs only." type="list" errorStyle="stop">
       <formula1>"ancient-worlds,gentle-nature,cosmic-journeys,cozy-tales"</formula1>
     </dataValidation>
-    <dataValidation sqref="J5:J62" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Rejected" error="Not an allowed value. Pick from the list." promptTitle="genreID_2" prompt="Existing genre IDs only." type="list" errorStyle="stop">
+    <dataValidation sqref="J5:J64" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Rejected" error="Not an allowed value. Pick from the list." promptTitle="genreID_2" prompt="Existing genre IDs only." type="list" errorStyle="stop">
       <formula1>"ancient-worlds,gentle-nature,cosmic-journeys,cozy-tales"</formula1>
     </dataValidation>
-    <dataValidation sqref="X5:X62" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Rejected" error="Not an allowed value. Pick from the list." promptTitle="commercialRightsStatus" prompt="Must be verified to publish." type="list" errorStyle="stop">
+    <dataValidation sqref="X5:X64" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Rejected" error="Not an allowed value. Pick from the list." promptTitle="commercialRightsStatus" prompt="Must be verified to publish." type="list" errorStyle="stop">
       <formula1>"pending-verification,verified,restricted"</formula1>
     </dataValidation>
-    <dataValidation sqref="K5:K62" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Rejected" error="Not an allowed value. Pick from the list." promptTitle="trialPreviewEligible" prompt="true or false." type="list" errorStyle="stop">
+    <dataValidation sqref="K5:K64" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Rejected" error="Not an allowed value. Pick from the list." promptTitle="trialPreviewEligible" prompt="true or false." type="list" errorStyle="stop">
       <formula1>"true,false"</formula1>
     </dataValidation>
-    <dataValidation sqref="L5:L62" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Rejected" error="Not an allowed value. Pick from the list." promptTitle="isFeatured" prompt="true or false." type="list" errorStyle="stop">
+    <dataValidation sqref="L5:L64" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Rejected" error="Not an allowed value. Pick from the list." promptTitle="isFeatured" prompt="true or false." type="list" errorStyle="stop">
       <formula1>"true,false"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
fix(pipeline): closeout now resets stale QA approval when audio bytes change
Found while reviewing the tracker for publish-readiness: the-rings-of-saturn
still carried its 2026-08-14 QA approval after being closed out against the
new Amy/Polly render on 2026-08-20 — closeout never touched the qa block, so
G13 was reporting PASS for audio nobody had actually listened to.

closeout now compares the incoming delivery checksum against what was on
record; if it differs and the story was already approved, it resets
audioApproved/deviceAccepted and prints a loud warning that re-listening is
required. Corrected the-rings-of-saturn's manifest by hand since its
staleness happened before this fix existed (checksums already matched by
the time the fix landed, so a second closeout run wouldn't have caught it).

Net effect: 0 of 26 stories are publish-ready until a human actually
listens to the current audio and runs `approve` — which is correct.
</commit_message>
<xml_diff>
--- a/Lullable_Story_Card_Tracker.xlsx
+++ b/Lullable_Story_Card_Tracker.xlsx
@@ -6202,7 +6202,7 @@
       </c>
       <c r="AA28" s="9" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>NOT READY</t>
         </is>
       </c>
       <c r="AB28" s="9" t="inlineStr">
@@ -6267,7 +6267,7 @@
       </c>
       <c r="AN28" s="9" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="AO28" s="9" t="inlineStr">

</xml_diff>

<commit_message>
content: credit four stories to Lullable, not to invented narrators
Bakery, Deep Ocean Trenches, Great Library and Ben Nevis now read
"Lullable" instead of the cast personas. Founder decision 2026-08-21,
these four only; the other 22 keep their casting.yaml credits.

casting.yaml is untouched and still drives which Polly voice renders each
category. This changes only what the listener is told, not what they hear.

Published and verified in staging: all four 18/18 gates, rows match the
manifests. Production promote pending founder approval.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Lullable_Story_Card_Tracker.xlsx
+++ b/Lullable_Story_Card_Tracker.xlsx
@@ -1292,7 +1292,7 @@
       </c>
       <c r="AO5" s="9" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AP5" s="9" t="inlineStr">
@@ -1371,7 +1371,7 @@
       </c>
       <c r="L6" s="7" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="M6" s="7" t="inlineStr">
@@ -1514,7 +1514,7 @@
       </c>
       <c r="AO6" s="9" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AP6" s="9" t="inlineStr">
@@ -1736,7 +1736,7 @@
       </c>
       <c r="AO7" s="9" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AP7" s="9" t="inlineStr">
@@ -1958,7 +1958,7 @@
       </c>
       <c r="AO8" s="9" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AP8" s="9" t="inlineStr">
@@ -2180,7 +2180,7 @@
       </c>
       <c r="AO9" s="9" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AP9" s="9" t="inlineStr">
@@ -2243,7 +2243,7 @@
       </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>Read by Niamh from Kinsale</t>
+          <t>Lullable</t>
         </is>
       </c>
       <c r="I10" s="7" t="inlineStr">
@@ -2402,7 +2402,7 @@
       </c>
       <c r="AO10" s="9" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AP10" s="9" t="inlineStr">
@@ -2624,7 +2624,7 @@
       </c>
       <c r="AO11" s="9" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AP11" s="9" t="inlineStr">
@@ -2846,7 +2846,7 @@
       </c>
       <c r="AO12" s="9" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AP12" s="9" t="inlineStr">
@@ -3068,7 +3068,7 @@
       </c>
       <c r="AO13" s="9" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AP13" s="9" t="inlineStr">
@@ -3131,7 +3131,7 @@
       </c>
       <c r="H14" s="7" t="inlineStr">
         <is>
-          <t>Read by Brian from St Ives</t>
+          <t>Lullable</t>
         </is>
       </c>
       <c r="I14" s="7" t="inlineStr">
@@ -3290,7 +3290,7 @@
       </c>
       <c r="AO14" s="9" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AP14" s="9" t="inlineStr">
@@ -3353,7 +3353,7 @@
       </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>Read by Arthur from Ludlow</t>
+          <t>Lullable</t>
         </is>
       </c>
       <c r="I15" s="7" t="inlineStr">
@@ -3512,7 +3512,7 @@
       </c>
       <c r="AO15" s="9" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AP15" s="9" t="inlineStr">
@@ -3956,7 +3956,7 @@
       </c>
       <c r="AO17" s="9" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AP17" s="9" t="inlineStr">
@@ -4178,7 +4178,7 @@
       </c>
       <c r="AO18" s="9" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AP18" s="9" t="inlineStr">
@@ -4400,7 +4400,7 @@
       </c>
       <c r="AO19" s="9" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AP19" s="9" t="inlineStr">
@@ -4622,7 +4622,7 @@
       </c>
       <c r="AO20" s="9" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AP20" s="9" t="inlineStr">
@@ -4844,7 +4844,7 @@
       </c>
       <c r="AO21" s="9" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AP21" s="9" t="inlineStr">
@@ -5066,7 +5066,7 @@
       </c>
       <c r="AO22" s="9" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AP22" s="9" t="inlineStr">
@@ -5288,7 +5288,7 @@
       </c>
       <c r="AO23" s="9" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AP23" s="9" t="inlineStr">
@@ -5510,7 +5510,7 @@
       </c>
       <c r="AO24" s="9" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AP24" s="9" t="inlineStr">
@@ -5732,7 +5732,7 @@
       </c>
       <c r="AO25" s="9" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AP25" s="9" t="inlineStr">
@@ -5795,7 +5795,7 @@
       </c>
       <c r="H26" s="7" t="inlineStr">
         <is>
-          <t>Read by Patrick, Block Island</t>
+          <t>Lullable</t>
         </is>
       </c>
       <c r="I26" s="7" t="inlineStr">
@@ -5954,7 +5954,7 @@
       </c>
       <c r="AO26" s="9" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AP26" s="9" t="inlineStr">
@@ -6176,7 +6176,7 @@
       </c>
       <c r="AO27" s="9" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AP27" s="9" t="inlineStr">
@@ -6255,7 +6255,7 @@
       </c>
       <c r="L28" s="7" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>false</t>
         </is>
       </c>
       <c r="M28" s="7" t="inlineStr">
@@ -6398,7 +6398,7 @@
       </c>
       <c r="AO28" s="9" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AP28" s="9" t="inlineStr">
@@ -6620,7 +6620,7 @@
       </c>
       <c r="AO29" s="9" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AP29" s="9" t="inlineStr">
@@ -6842,7 +6842,7 @@
       </c>
       <c r="AO30" s="9" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AP30" s="9" t="inlineStr">

</xml_diff>